<commit_message>
Atualização automática da planilha
</commit_message>
<xml_diff>
--- a/template-softexpert.xlsx
+++ b/template-softexpert.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://planoeplano-my.sharepoint.com/personal/lucas_fernandes_planoeplano_com_br/Documents/Área de Trabalho/Softexpert/Teste/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="450" documentId="11_C24A341F8ED520438A3C56126D326013BF438F93" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DEA9788-5B69-4CF1-B047-0DA09974B374}"/>
+  <xr:revisionPtr revIDLastSave="453" documentId="11_C24A341F8ED520438A3C56126D326013BF438F93" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{08866576-0D57-483C-ADAA-AD6B8671A834}"/>
   <bookViews>
-    <workbookView xWindow="2660" yWindow="2660" windowWidth="14400" windowHeight="8170" tabRatio="500" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2660" yWindow="2660" windowWidth="14400" windowHeight="8170" tabRatio="500" firstSheet="2" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Programa" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1385" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="314">
   <si>
     <t>Campo</t>
   </si>
@@ -485,502 +485,343 @@
     <t>Aberto / Mitigando / Bloqueado / Em tratamento / Pendente / Concluído</t>
   </si>
   <si>
-    <t>R01</t>
-  </si>
-  <si>
-    <t>Risco</t>
-  </si>
-  <si>
-    <t>Atraso na alocação de key users de Riscos</t>
-  </si>
-  <si>
-    <t>Gestão de Riscos</t>
-  </si>
-  <si>
-    <t>Alto</t>
-  </si>
-  <si>
-    <t>Cronograma</t>
-  </si>
-  <si>
-    <t>Solicitar reforço via Presidência</t>
-  </si>
-  <si>
-    <t>Aberto</t>
-  </si>
-  <si>
-    <t>10/01/2026</t>
-  </si>
-  <si>
-    <t>R02</t>
-  </si>
-  <si>
-    <t>Integração com ERP legado (SAP) com escopo indefinido</t>
-  </si>
-  <si>
-    <t>Gestão de Processos (BPM)</t>
-  </si>
-  <si>
-    <t>Escopo</t>
-  </si>
-  <si>
-    <t>Workshop técnico agendado para 18/02</t>
-  </si>
-  <si>
-    <t>Thiago Gomes</t>
-  </si>
-  <si>
-    <t>15/01/2026</t>
-  </si>
-  <si>
-    <t>I01</t>
-  </si>
-  <si>
-    <t>Impedimento</t>
-  </si>
-  <si>
-    <t>Aprovação de orçamento para licenças de Fornecedores</t>
-  </si>
-  <si>
-    <t>Gestão de Fornecedores</t>
-  </si>
-  <si>
-    <t>Crítico</t>
-  </si>
-  <si>
-    <t>Custo</t>
-  </si>
-  <si>
-    <t>Aguardando aprovação da Presidência</t>
-  </si>
-  <si>
-    <t>Diretoria Financeira</t>
-  </si>
-  <si>
-    <t>Bloqueado</t>
-  </si>
-  <si>
-    <t>20/01/2026</t>
-  </si>
-  <si>
-    <t>I02</t>
-  </si>
-  <si>
-    <t>Ambiente de homologação com performance degradada</t>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>% Avanço Geral</t>
+  </si>
+  <si>
+    <t>Média dos projetos (0-100)</t>
+  </si>
+  <si>
+    <t>Nível</t>
+  </si>
+  <si>
+    <t>Papel</t>
+  </si>
+  <si>
+    <t>Cargo / Título</t>
+  </si>
+  <si>
+    <t>Sponsor / Comitê Exec. / Gestão / Líder Arq. / Decisor Go-NoGo / Time Projeto</t>
+  </si>
+  <si>
+    <t>Papel no programa</t>
+  </si>
+  <si>
+    <t>Nome completo</t>
+  </si>
+  <si>
+    <t>Cargo na empresa</t>
+  </si>
+  <si>
+    <t>Área de negócio</t>
+  </si>
+  <si>
+    <t>Sponsor</t>
+  </si>
+  <si>
+    <t>Sponsor Executivo</t>
+  </si>
+  <si>
+    <t>Rodrigo Fairbanks von Uhlendorff</t>
+  </si>
+  <si>
+    <t>Presidente</t>
+  </si>
+  <si>
+    <t>Presidência</t>
+  </si>
+  <si>
+    <t>Comitê Executivo</t>
+  </si>
+  <si>
+    <t>Membro do Comitê</t>
+  </si>
+  <si>
+    <t>Henrique Hildebrand Garcia</t>
+  </si>
+  <si>
+    <t>Diretor Jurídico</t>
+  </si>
+  <si>
+    <t>Leonardo Araujo</t>
+  </si>
+  <si>
+    <t>Diretor De Operacoes Financeiras e TI</t>
+  </si>
+  <si>
+    <t>Operacoes Financeiras e TI</t>
+  </si>
+  <si>
+    <t>Marco Cardoso</t>
+  </si>
+  <si>
+    <t>Superintendente de TI</t>
+  </si>
+  <si>
+    <t>Tecnologia da Informação</t>
+  </si>
+  <si>
+    <t>Renee Silveira</t>
+  </si>
+  <si>
+    <t>Diretora De Incorporação</t>
+  </si>
+  <si>
+    <t>Gestão do Programa</t>
+  </si>
+  <si>
+    <t>Gerente de Projetos</t>
+  </si>
+  <si>
+    <t>Fabio Jonas</t>
+  </si>
+  <si>
+    <t>Gerente De Riscos E Controles Internos</t>
+  </si>
+  <si>
+    <t>Fernando Hideo Fujii</t>
+  </si>
+  <si>
+    <t>Gerente de Programa</t>
+  </si>
+  <si>
+    <t>Coordenador de Sistemas</t>
+  </si>
+  <si>
+    <t>Claudio Ferreira</t>
+  </si>
+  <si>
+    <t>DBD - Gerente de Projetos</t>
+  </si>
+  <si>
+    <t>DBD</t>
+  </si>
+  <si>
+    <t>Leonardo Bazzo Scurupa</t>
+  </si>
+  <si>
+    <t>SoftExpert - Gerente de Projetos</t>
+  </si>
+  <si>
+    <t>SoftExpert</t>
+  </si>
+  <si>
+    <t>Líder Arquitetura/Infra</t>
+  </si>
+  <si>
+    <t>Líder de Arquitetura</t>
+  </si>
+  <si>
+    <t>Marco Andres Quezada</t>
+  </si>
+  <si>
+    <t>Gerente de Infraestrutura</t>
+  </si>
+  <si>
+    <t>Rodrigo Bernardo</t>
+  </si>
+  <si>
+    <t>Decisor Go-NoGo</t>
+  </si>
+  <si>
+    <t>Gerente de Sistemas</t>
+  </si>
+  <si>
+    <t>Luiz Antonio Novaes</t>
+  </si>
+  <si>
+    <t>Líderes de Negócios</t>
+  </si>
+  <si>
+    <t>Time Projeto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analista de Sistemas </t>
+  </si>
+  <si>
+    <t>Luciano da Rocha Rafael</t>
+  </si>
+  <si>
+    <t>Vinicius França Nascimento</t>
+  </si>
+  <si>
+    <t>Líder de Projeto</t>
+  </si>
+  <si>
+    <t>Andreza Benatti</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consultor </t>
+  </si>
+  <si>
+    <t>Marcelo Ferreira</t>
+  </si>
+  <si>
+    <t>Consultor Projeto: Engenharia</t>
+  </si>
+  <si>
+    <t>Andre Sterzza</t>
+  </si>
+  <si>
+    <t>Consultor Projeto: Contratos</t>
+  </si>
+  <si>
+    <t>Cristian Quadros</t>
+  </si>
+  <si>
+    <t>Consultor Projeto: Contas a Receber</t>
+  </si>
+  <si>
+    <t>Daiane Leite</t>
+  </si>
+  <si>
+    <t>Consultor Projeto: TI/ITSM/GMUD</t>
+  </si>
+  <si>
+    <t>Dany Zoboli</t>
+  </si>
+  <si>
+    <t>Consultor Projeto: Core Business; Captação; Contratação</t>
+  </si>
+  <si>
+    <t>Donato de Avila</t>
+  </si>
+  <si>
+    <t>Consultor Projeto:GRC; Auditoria Interna</t>
+  </si>
+  <si>
+    <t>Janaina Azevedo</t>
+  </si>
+  <si>
+    <t>Consultor Projeto: Portal do Fornecedor; Qualidade</t>
+  </si>
+  <si>
+    <t>Neimar Carvalho</t>
+  </si>
+  <si>
+    <t>Key User N1</t>
+  </si>
+  <si>
+    <t>Mayara Santos</t>
+  </si>
+  <si>
+    <t>Coordenadora De Novos Negocios</t>
+  </si>
+  <si>
+    <t>Key User N2</t>
+  </si>
+  <si>
+    <t>Laura Barbosa Ribeiro</t>
+  </si>
+  <si>
+    <t>Assistente de Novos Negócios</t>
+  </si>
+  <si>
+    <t>Gina De Giuseppe</t>
+  </si>
+  <si>
+    <t>Coordenadora De Incorporacao</t>
+  </si>
+  <si>
+    <t>Luciana Vieira</t>
+  </si>
+  <si>
+    <t>Gerente de Incorporação</t>
+  </si>
+  <si>
+    <t>Adriana Bittencourt</t>
+  </si>
+  <si>
+    <t>Gerente Jurídico</t>
+  </si>
+  <si>
+    <t>Alexandre Tavares de Gouvea</t>
+  </si>
+  <si>
+    <t>Gabriela Costa do Nascimento</t>
+  </si>
+  <si>
+    <t>Advogado SR</t>
+  </si>
+  <si>
+    <t>Pedro Henrique de Oliveira</t>
+  </si>
+  <si>
+    <t>SLO - Terceiro</t>
+  </si>
+  <si>
+    <t>Tadashi Sato</t>
+  </si>
+  <si>
+    <t>Luciana de Carvalho Cavalcante</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coordenadora Juridico  </t>
+  </si>
+  <si>
+    <t>Eduardo Cerri</t>
+  </si>
+  <si>
+    <t> </t>
+  </si>
+  <si>
+    <t>Planejamento e Relação com Investidores</t>
+  </si>
+  <si>
+    <t>Rodrigo Kawakami</t>
+  </si>
+  <si>
+    <t>Vanessa Kato</t>
+  </si>
+  <si>
+    <t>Stand</t>
+  </si>
+  <si>
+    <t>Superintendente</t>
+  </si>
+  <si>
+    <t>Marcos Souza</t>
+  </si>
+  <si>
+    <t>Viabilidade Economica</t>
+  </si>
+  <si>
+    <t>Adriana Brasca Raposo</t>
+  </si>
+  <si>
+    <t>Bruna Fernandes</t>
+  </si>
+  <si>
+    <t>Aprovações</t>
+  </si>
+  <si>
+    <t>Elmo Kanashiro</t>
+  </si>
+  <si>
+    <t>Fabiana Passos</t>
+  </si>
+  <si>
+    <t>Inteligência de Mercado</t>
+  </si>
+  <si>
+    <t>Sagar Kuzhiparambil Prakasan</t>
+  </si>
+  <si>
+    <t>Sandra Trombeli</t>
+  </si>
+  <si>
+    <t>Projetos</t>
+  </si>
+  <si>
+    <t>Paulo Gambini</t>
+  </si>
+  <si>
+    <t>Carlos Morais</t>
   </si>
   <si>
     <t>Infraestrutura</t>
-  </si>
-  <si>
-    <t>Médio</t>
-  </si>
-  <si>
-    <t>Ticket aberto com Softexpert</t>
-  </si>
-  <si>
-    <t>Rafael Nunes</t>
-  </si>
-  <si>
-    <t>Em tratamento</t>
-  </si>
-  <si>
-    <t>03/02/2026</t>
-  </si>
-  <si>
-    <t>I03</t>
-  </si>
-  <si>
-    <t>Taxonomia corporativa de processos pendente</t>
-  </si>
-  <si>
-    <t>Comitê de Processos em definição</t>
-  </si>
-  <si>
-    <t>D09</t>
-  </si>
-  <si>
-    <t>Decisão</t>
-  </si>
-  <si>
-    <t>Aprovar alocação de 2 recursos adicionais do time de TI para Gestão de Riscos</t>
-  </si>
-  <si>
-    <t>Presidência</t>
-  </si>
-  <si>
-    <t>20/02/2026</t>
-  </si>
-  <si>
-    <t> </t>
-  </si>
-  <si>
-    <t>D10</t>
-  </si>
-  <si>
-    <t>Definir prioridade entre Indicadores e Fornecedores para alocação de key users Q2</t>
-  </si>
-  <si>
-    <t>28/02/2026</t>
-  </si>
-  <si>
-    <t>D11</t>
-  </si>
-  <si>
-    <t>Validar orçamento adicional de R$ 85K para treinamentos avançados Softexpert</t>
-  </si>
-  <si>
-    <t>15/03/2026</t>
-  </si>
-  <si>
-    <t>C01</t>
-  </si>
-  <si>
-    <t>Conquista</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kanban Qualidade - Permite que a área faça gestão das atividades do time através da solução. </t>
-  </si>
-  <si>
-    <t>11/02/2026</t>
-  </si>
-  <si>
-    <t>C02</t>
-  </si>
-  <si>
-    <t>Implementação de SSO – Permite que o usuário acesse o sistema automaticamente, usando o mesmo login que já está conectado na sua máquina, sem precisar digitar senha novamente.</t>
-  </si>
-  <si>
-    <t>30/01/2026</t>
-  </si>
-  <si>
-    <t>Data</t>
-  </si>
-  <si>
-    <t>% Avanço Geral</t>
-  </si>
-  <si>
-    <t>Média dos projetos (0-100)</t>
-  </si>
-  <si>
-    <t>Nível</t>
-  </si>
-  <si>
-    <t>Papel</t>
-  </si>
-  <si>
-    <t>Cargo / Título</t>
-  </si>
-  <si>
-    <t>Sponsor / Comitê Exec. / Gestão / Líder Arq. / Decisor Go-NoGo / Time Projeto</t>
-  </si>
-  <si>
-    <t>Papel no programa</t>
-  </si>
-  <si>
-    <t>Nome completo</t>
-  </si>
-  <si>
-    <t>Cargo na empresa</t>
-  </si>
-  <si>
-    <t>Área de negócio</t>
-  </si>
-  <si>
-    <t>Sponsor</t>
-  </si>
-  <si>
-    <t>Sponsor Executivo</t>
-  </si>
-  <si>
-    <t>Rodrigo Fairbanks von Uhlendorff</t>
-  </si>
-  <si>
-    <t>Presidente</t>
-  </si>
-  <si>
-    <t>Comitê Executivo</t>
-  </si>
-  <si>
-    <t>Membro do Comitê</t>
-  </si>
-  <si>
-    <t>Henrique Hildebrand Garcia</t>
-  </si>
-  <si>
-    <t>Diretor Jurídico</t>
-  </si>
-  <si>
-    <t>Leonardo Araujo</t>
-  </si>
-  <si>
-    <t>Diretor De Operacoes Financeiras e TI</t>
-  </si>
-  <si>
-    <t>Operacoes Financeiras e TI</t>
-  </si>
-  <si>
-    <t>Marco Cardoso</t>
-  </si>
-  <si>
-    <t>Superintendente de TI</t>
-  </si>
-  <si>
-    <t>Tecnologia da Informação</t>
-  </si>
-  <si>
-    <t>Renee Silveira</t>
-  </si>
-  <si>
-    <t>Diretora De Incorporação</t>
-  </si>
-  <si>
-    <t>Gestão do Programa</t>
-  </si>
-  <si>
-    <t>Gerente de Projetos</t>
-  </si>
-  <si>
-    <t>Fabio Jonas</t>
-  </si>
-  <si>
-    <t>Gerente De Riscos E Controles Internos</t>
-  </si>
-  <si>
-    <t>Fernando Hideo Fujii</t>
-  </si>
-  <si>
-    <t>Gerente de Programa</t>
-  </si>
-  <si>
-    <t>Coordenador de Sistemas</t>
-  </si>
-  <si>
-    <t>Claudio Ferreira</t>
-  </si>
-  <si>
-    <t>DBD - Gerente de Projetos</t>
-  </si>
-  <si>
-    <t>DBD</t>
-  </si>
-  <si>
-    <t>Leonardo Bazzo Scurupa</t>
-  </si>
-  <si>
-    <t>SoftExpert - Gerente de Projetos</t>
-  </si>
-  <si>
-    <t>SoftExpert</t>
-  </si>
-  <si>
-    <t>Líder Arquitetura/Infra</t>
-  </si>
-  <si>
-    <t>Líder de Arquitetura</t>
-  </si>
-  <si>
-    <t>Marco Andres Quezada</t>
-  </si>
-  <si>
-    <t>Gerente de Infraestrutura</t>
-  </si>
-  <si>
-    <t>Rodrigo Bernardo</t>
-  </si>
-  <si>
-    <t>Decisor Go-NoGo</t>
-  </si>
-  <si>
-    <t>Gerente de Sistemas</t>
-  </si>
-  <si>
-    <t>Luiz Antonio Novaes</t>
-  </si>
-  <si>
-    <t>Líderes de Negócios</t>
-  </si>
-  <si>
-    <t>Time Projeto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Analista de Sistemas </t>
-  </si>
-  <si>
-    <t>Luciano da Rocha Rafael</t>
-  </si>
-  <si>
-    <t>Vinicius França Nascimento</t>
-  </si>
-  <si>
-    <t>Líder de Projeto</t>
-  </si>
-  <si>
-    <t>Andreza Benatti</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consultor </t>
-  </si>
-  <si>
-    <t>Marcelo Ferreira</t>
-  </si>
-  <si>
-    <t>Consultor Projeto: Engenharia</t>
-  </si>
-  <si>
-    <t>Andre Sterzza</t>
-  </si>
-  <si>
-    <t>Consultor Projeto: Contratos</t>
-  </si>
-  <si>
-    <t>Cristian Quadros</t>
-  </si>
-  <si>
-    <t>Consultor Projeto: Contas a Receber</t>
-  </si>
-  <si>
-    <t>Daiane Leite</t>
-  </si>
-  <si>
-    <t>Consultor Projeto: TI/ITSM/GMUD</t>
-  </si>
-  <si>
-    <t>Dany Zoboli</t>
-  </si>
-  <si>
-    <t>Consultor Projeto: Core Business; Captação; Contratação</t>
-  </si>
-  <si>
-    <t>Donato de Avila</t>
-  </si>
-  <si>
-    <t>Consultor Projeto:GRC; Auditoria Interna</t>
-  </si>
-  <si>
-    <t>Janaina Azevedo</t>
-  </si>
-  <si>
-    <t>Consultor Projeto: Portal do Fornecedor; Qualidade</t>
-  </si>
-  <si>
-    <t>Neimar Carvalho</t>
-  </si>
-  <si>
-    <t>Key User N1</t>
-  </si>
-  <si>
-    <t>Mayara Santos</t>
-  </si>
-  <si>
-    <t>Coordenadora De Novos Negocios</t>
-  </si>
-  <si>
-    <t>Key User N2</t>
-  </si>
-  <si>
-    <t>Laura Barbosa Ribeiro</t>
-  </si>
-  <si>
-    <t>Assistente de Novos Negócios</t>
-  </si>
-  <si>
-    <t>Gina De Giuseppe</t>
-  </si>
-  <si>
-    <t>Coordenadora De Incorporacao</t>
-  </si>
-  <si>
-    <t>Luciana Vieira</t>
-  </si>
-  <si>
-    <t>Gerente de Incorporação</t>
-  </si>
-  <si>
-    <t>Adriana Bittencourt</t>
-  </si>
-  <si>
-    <t>Gerente Jurídico</t>
-  </si>
-  <si>
-    <t>Alexandre Tavares de Gouvea</t>
-  </si>
-  <si>
-    <t>Gabriela Costa do Nascimento</t>
-  </si>
-  <si>
-    <t>Advogado SR</t>
-  </si>
-  <si>
-    <t>Pedro Henrique de Oliveira</t>
-  </si>
-  <si>
-    <t>SLO - Terceiro</t>
-  </si>
-  <si>
-    <t>Tadashi Sato</t>
-  </si>
-  <si>
-    <t>Luciana de Carvalho Cavalcante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coordenadora Juridico  </t>
-  </si>
-  <si>
-    <t>Eduardo Cerri</t>
-  </si>
-  <si>
-    <t>Planejamento e Relação com Investidores</t>
-  </si>
-  <si>
-    <t>Rodrigo Kawakami</t>
-  </si>
-  <si>
-    <t>Vanessa Kato</t>
-  </si>
-  <si>
-    <t>Stand</t>
-  </si>
-  <si>
-    <t>Superintendente</t>
-  </si>
-  <si>
-    <t>Marcos Souza</t>
-  </si>
-  <si>
-    <t>Viabilidade Economica</t>
-  </si>
-  <si>
-    <t>Adriana Brasca Raposo</t>
-  </si>
-  <si>
-    <t>Bruna Fernandes</t>
-  </si>
-  <si>
-    <t>Aprovações</t>
-  </si>
-  <si>
-    <t>Elmo Kanashiro</t>
-  </si>
-  <si>
-    <t>Fabiana Passos</t>
-  </si>
-  <si>
-    <t>Inteligência de Mercado</t>
-  </si>
-  <si>
-    <t>Sagar Kuzhiparambil Prakasan</t>
-  </si>
-  <si>
-    <t>Sandra Trombeli</t>
-  </si>
-  <si>
-    <t>Projetos</t>
-  </si>
-  <si>
-    <t>Paulo Gambini</t>
-  </si>
-  <si>
-    <t>Carlos Morais</t>
   </si>
   <si>
     <t>Silvia Reis</t>
@@ -1168,7 +1009,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="m/d/yyyy"/>
-    <numFmt numFmtId="166" formatCode="&quot;R$&quot;\ #,##0.00"/>
+    <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="14">
     <font>
@@ -1502,7 +1343,7 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
@@ -1809,7 +1650,7 @@
       </c>
       <c r="B4" s="12" t="str">
         <f ca="1">TEXT(NOW(),"DD/MM/AAAA")</f>
-        <v>20/02/2026</v>
+        <v>23/02/2026</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1">
@@ -1878,13 +1719,13 @@
         <v>132</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>355</v>
+        <v>302</v>
       </c>
       <c r="C1" s="35" t="s">
         <v>69</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>356</v>
+        <v>303</v>
       </c>
       <c r="E1" s="36">
         <v>45992</v>
@@ -1928,66 +1769,66 @@
     </row>
     <row r="2" spans="1:17" ht="14.25" customHeight="1">
       <c r="A2" s="30" t="s">
-        <v>357</v>
+        <v>304</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>358</v>
+        <v>305</v>
       </c>
       <c r="C2" s="31" t="s">
         <v>71</v>
       </c>
       <c r="D2" s="31" t="s">
-        <v>359</v>
+        <v>306</v>
       </c>
       <c r="E2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="F2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="G2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="H2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="I2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="J2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="K2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="L2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="M2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="N2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="O2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="P2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="Q2" s="31" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
     </row>
     <row r="3" spans="1:17" ht="14.25" customHeight="1">
       <c r="A3" s="37" t="s">
-        <v>360</v>
+        <v>307</v>
       </c>
       <c r="B3" s="38" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
       <c r="C3" s="38" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="D3" s="39">
         <v>50000</v>
@@ -2012,10 +1853,10 @@
     </row>
     <row r="4" spans="1:17" ht="14.25" customHeight="1">
       <c r="A4" s="37" t="s">
-        <v>361</v>
+        <v>308</v>
       </c>
       <c r="B4" s="38" t="s">
-        <v>235</v>
+        <v>180</v>
       </c>
       <c r="C4" s="38" t="s">
         <v>26</v>
@@ -2047,10 +1888,10 @@
     </row>
     <row r="5" spans="1:17" ht="14.25" customHeight="1">
       <c r="A5" s="37" t="s">
-        <v>362</v>
+        <v>309</v>
       </c>
       <c r="B5" s="38" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
       <c r="C5" s="38"/>
       <c r="D5" s="39">
@@ -2074,10 +1915,10 @@
     </row>
     <row r="6" spans="1:17" ht="14.25" customHeight="1">
       <c r="A6" s="37" t="s">
-        <v>362</v>
+        <v>309</v>
       </c>
       <c r="B6" s="38" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
       <c r="C6" s="38" t="s">
         <v>31</v>
@@ -2101,10 +1942,10 @@
     </row>
     <row r="7" spans="1:17" ht="14.25" customHeight="1">
       <c r="A7" s="37" t="s">
-        <v>171</v>
+        <v>255</v>
       </c>
       <c r="B7" s="38" t="s">
-        <v>363</v>
+        <v>310</v>
       </c>
       <c r="C7" s="38" t="s">
         <v>37</v>
@@ -2130,13 +1971,13 @@
     </row>
     <row r="8" spans="1:17" ht="15" customHeight="1">
       <c r="A8" s="37" t="s">
-        <v>364</v>
+        <v>311</v>
       </c>
       <c r="B8" s="38" t="s">
-        <v>365</v>
+        <v>312</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="D8" s="39">
         <v>0</v>
@@ -2157,13 +1998,13 @@
     </row>
     <row r="9" spans="1:17" ht="15" customHeight="1">
       <c r="A9" s="37" t="s">
-        <v>366</v>
+        <v>313</v>
       </c>
       <c r="B9" s="38" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="D9" s="39">
         <v>0</v>
@@ -2184,10 +2025,10 @@
     </row>
     <row r="10" spans="1:17" ht="27.75" customHeight="1">
       <c r="A10" s="37" t="s">
-        <v>171</v>
+        <v>255</v>
       </c>
       <c r="B10" s="38" t="s">
-        <v>363</v>
+        <v>310</v>
       </c>
       <c r="C10" s="38" t="s">
         <v>37</v>
@@ -2336,7 +2177,9 @@
       <c r="B3" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="14"/>
+      <c r="C3" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="D3" s="14" t="s">
         <v>28</v>
       </c>
@@ -2369,7 +2212,9 @@
       <c r="B4" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C4" s="14"/>
+      <c r="C4" s="14" t="s">
+        <v>32</v>
+      </c>
       <c r="D4" s="14" t="s">
         <v>28</v>
       </c>
@@ -5412,331 +5257,143 @@
       </c>
     </row>
     <row r="3" spans="1:12" ht="35.1" customHeight="1">
-      <c r="A3" s="14" t="s">
-        <v>143</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>145</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>146</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>149</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>125</v>
-      </c>
-      <c r="J3" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>151</v>
-      </c>
-      <c r="L3" s="40">
-        <v>46096</v>
-      </c>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="40"/>
     </row>
     <row r="4" spans="1:12" ht="24.75" customHeight="1">
-      <c r="A4" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>144</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>153</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="F4" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="I4" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="J4" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="K4" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="L4" s="32">
-        <v>46081</v>
-      </c>
+      <c r="A4" s="14"/>
+      <c r="B4" s="14"/>
+      <c r="C4" s="14"/>
+      <c r="D4" s="14"/>
+      <c r="E4" s="14"/>
+      <c r="F4" s="14"/>
+      <c r="G4" s="14"/>
+      <c r="H4" s="14"/>
+      <c r="I4" s="14"/>
+      <c r="J4" s="14"/>
+      <c r="K4" s="14"/>
+      <c r="L4" s="32"/>
     </row>
     <row r="5" spans="1:12" ht="24.75" customHeight="1">
-      <c r="A5" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>161</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>147</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>165</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>166</v>
-      </c>
-      <c r="J5" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="K5" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="L5" s="32">
-        <v>46122</v>
-      </c>
+      <c r="A5" s="14"/>
+      <c r="B5" s="14"/>
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+      <c r="G5" s="14"/>
+      <c r="H5" s="14"/>
+      <c r="I5" s="14"/>
+      <c r="J5" s="14"/>
+      <c r="K5" s="14"/>
+      <c r="L5" s="32"/>
     </row>
     <row r="6" spans="1:12" ht="24.75" customHeight="1">
-      <c r="A6" s="14" t="s">
-        <v>169</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>171</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>148</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="I6" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="J6" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="K6" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="L6" s="32">
-        <v>46082</v>
-      </c>
+      <c r="A6" s="14"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+      <c r="L6" s="32"/>
     </row>
     <row r="7" spans="1:12" ht="46.35" customHeight="1">
-      <c r="A7" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>178</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>154</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>172</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>179</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>124</v>
-      </c>
-      <c r="J7" s="14" t="s">
-        <v>175</v>
-      </c>
-      <c r="K7" s="14" t="s">
-        <v>158</v>
-      </c>
-      <c r="L7" s="32">
-        <v>46101</v>
-      </c>
+      <c r="A7" s="14"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="14"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="14"/>
+      <c r="J7" s="14"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="32"/>
     </row>
     <row r="8" spans="1:12" ht="57.6" customHeight="1">
-      <c r="A8" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="B8" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>182</v>
-      </c>
+      <c r="A8" s="17"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="17"/>
       <c r="D8" s="17"/>
       <c r="E8" s="17"/>
       <c r="F8" s="17"/>
       <c r="G8" s="17"/>
       <c r="H8" s="17"/>
-      <c r="I8" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="J8" s="17" t="s">
-        <v>121</v>
-      </c>
-      <c r="K8" s="17" t="s">
-        <v>184</v>
-      </c>
-      <c r="L8" s="41" t="s">
-        <v>185</v>
-      </c>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17"/>
+      <c r="L8" s="41"/>
     </row>
     <row r="9" spans="1:12" ht="57.6" customHeight="1">
-      <c r="A9" s="17" t="s">
-        <v>186</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>187</v>
-      </c>
+      <c r="A9" s="17"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="17"/>
       <c r="E9" s="17"/>
       <c r="F9" s="17"/>
       <c r="G9" s="17"/>
       <c r="H9" s="17"/>
-      <c r="I9" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="J9" s="17" t="s">
-        <v>121</v>
-      </c>
-      <c r="K9" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="L9" s="41" t="s">
-        <v>185</v>
-      </c>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
+      <c r="K9" s="17"/>
+      <c r="L9" s="41"/>
     </row>
     <row r="10" spans="1:12" ht="68.650000000000006" customHeight="1">
-      <c r="A10" s="17" t="s">
-        <v>189</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>181</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>190</v>
-      </c>
+      <c r="A10" s="17"/>
+      <c r="B10" s="17"/>
+      <c r="C10" s="17"/>
       <c r="D10" s="17"/>
       <c r="E10" s="17"/>
       <c r="F10" s="17"/>
       <c r="G10" s="17"/>
       <c r="H10" s="17"/>
-      <c r="I10" s="17" t="s">
-        <v>183</v>
-      </c>
-      <c r="J10" s="17" t="s">
-        <v>121</v>
-      </c>
-      <c r="K10" s="17" t="s">
-        <v>191</v>
-      </c>
-      <c r="L10" s="32">
-        <v>46111</v>
-      </c>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
+      <c r="K10" s="17"/>
+      <c r="L10" s="32"/>
     </row>
     <row r="11" spans="1:12" ht="79.900000000000006" customHeight="1">
-      <c r="A11" s="17" t="s">
-        <v>192</v>
-      </c>
-      <c r="B11" s="17" t="s">
-        <v>193</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>194</v>
-      </c>
+      <c r="A11" s="17"/>
+      <c r="B11" s="17"/>
+      <c r="C11" s="17"/>
       <c r="D11" s="17"/>
       <c r="E11" s="17"/>
       <c r="F11" s="17"/>
       <c r="G11" s="17"/>
       <c r="H11" s="17"/>
-      <c r="I11" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="J11" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="K11" s="25" t="s">
-        <v>195</v>
-      </c>
-      <c r="L11" s="32">
-        <v>46127</v>
-      </c>
+      <c r="I11" s="17"/>
+      <c r="J11" s="24"/>
+      <c r="K11" s="25"/>
+      <c r="L11" s="32"/>
     </row>
     <row r="12" spans="1:12" ht="46.35" customHeight="1">
-      <c r="A12" s="17" t="s">
-        <v>196</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>193</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>197</v>
-      </c>
+      <c r="A12" s="17"/>
+      <c r="B12" s="17"/>
+      <c r="C12" s="17"/>
       <c r="D12" s="17"/>
       <c r="E12" s="17"/>
       <c r="F12" s="17"/>
       <c r="G12" s="17"/>
       <c r="H12" s="17"/>
-      <c r="I12" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="J12" s="24" t="s">
-        <v>77</v>
-      </c>
-      <c r="K12" s="25" t="s">
-        <v>198</v>
-      </c>
+      <c r="I12" s="17"/>
+      <c r="J12" s="24"/>
+      <c r="K12" s="25"/>
       <c r="L12" s="28"/>
     </row>
     <row r="13" spans="1:12" ht="15">
@@ -5768,10 +5425,10 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="26" t="s">
-        <v>199</v>
+        <v>143</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>200</v>
+        <v>144</v>
       </c>
       <c r="C1" s="28"/>
       <c r="D1" s="28"/>
@@ -5784,7 +5441,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="31" t="s">
-        <v>201</v>
+        <v>145</v>
       </c>
       <c r="C2" s="28"/>
       <c r="D2" s="28"/>
@@ -5984,16 +5641,16 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="9" t="s">
-        <v>202</v>
+        <v>146</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>203</v>
+        <v>147</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>117</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>204</v>
+        <v>148</v>
       </c>
       <c r="E1" s="9" t="s">
         <v>9</v>
@@ -6001,50 +5658,50 @@
     </row>
     <row r="2" spans="1:5" ht="66.75">
       <c r="A2" s="13" t="s">
-        <v>205</v>
+        <v>149</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>206</v>
+        <v>150</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>207</v>
+        <v>151</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>208</v>
+        <v>152</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>209</v>
+        <v>153</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="48">
       <c r="A3" s="14" t="s">
-        <v>210</v>
+        <v>154</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>211</v>
+        <v>155</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>212</v>
+        <v>156</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>213</v>
+        <v>157</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>183</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="36">
       <c r="A4" s="14" t="s">
-        <v>214</v>
+        <v>159</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>215</v>
+        <v>160</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>216</v>
+        <v>161</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>217</v>
+        <v>162</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>35</v>
@@ -6052,50 +5709,50 @@
     </row>
     <row r="5" spans="1:5" ht="36">
       <c r="A5" s="14" t="s">
-        <v>214</v>
+        <v>159</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>215</v>
+        <v>160</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>218</v>
+        <v>163</v>
       </c>
       <c r="D5" s="14" t="s">
-        <v>219</v>
+        <v>164</v>
       </c>
       <c r="E5" s="14" t="s">
-        <v>220</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="36">
       <c r="A6" s="14" t="s">
-        <v>214</v>
+        <v>159</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>215</v>
+        <v>160</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>221</v>
+        <v>166</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>222</v>
+        <v>167</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="24">
       <c r="A7" s="14" t="s">
-        <v>214</v>
+        <v>159</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>215</v>
+        <v>160</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>224</v>
+        <v>169</v>
       </c>
       <c r="D7" s="14" t="s">
-        <v>225</v>
+        <v>170</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>27</v>
@@ -6103,16 +5760,16 @@
     </row>
     <row r="8" spans="1:5" ht="36">
       <c r="A8" s="14" t="s">
-        <v>226</v>
+        <v>171</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>227</v>
+        <v>172</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>228</v>
+        <v>173</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>229</v>
+        <v>174</v>
       </c>
       <c r="E8" s="17" t="s">
         <v>39</v>
@@ -6120,374 +5777,374 @@
     </row>
     <row r="9" spans="1:5" ht="36">
       <c r="A9" s="14" t="s">
-        <v>226</v>
+        <v>171</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>227</v>
+        <v>172</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>230</v>
+        <v>175</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>227</v>
+        <v>172</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="36">
       <c r="A10" s="14" t="s">
-        <v>226</v>
+        <v>171</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>231</v>
+        <v>176</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>28</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>232</v>
+        <v>177</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="24">
       <c r="A11" s="14" t="s">
-        <v>226</v>
+        <v>171</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>227</v>
+        <v>172</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>233</v>
+        <v>178</v>
       </c>
       <c r="D11" s="14" t="s">
-        <v>234</v>
+        <v>179</v>
       </c>
       <c r="E11" s="14" t="s">
-        <v>235</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="36">
       <c r="A12" s="14" t="s">
-        <v>226</v>
+        <v>171</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>227</v>
+        <v>172</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>236</v>
+        <v>181</v>
       </c>
       <c r="D12" s="14" t="s">
-        <v>237</v>
+        <v>182</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="36">
       <c r="A13" s="14" t="s">
-        <v>239</v>
+        <v>184</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>240</v>
+        <v>185</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>241</v>
+        <v>186</v>
       </c>
       <c r="D13" s="14" t="s">
-        <v>240</v>
+        <v>185</v>
       </c>
       <c r="E13" s="14" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="36">
       <c r="A14" s="14" t="s">
-        <v>239</v>
+        <v>184</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>242</v>
+        <v>187</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>243</v>
+        <v>188</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>242</v>
+        <v>187</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="36">
       <c r="A15" s="14" t="s">
-        <v>244</v>
+        <v>189</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>245</v>
+        <v>190</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>246</v>
+        <v>191</v>
       </c>
       <c r="D15" s="14" t="s">
-        <v>245</v>
+        <v>190</v>
       </c>
       <c r="E15" s="14" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="24">
       <c r="A16" s="14" t="s">
-        <v>244</v>
+        <v>189</v>
       </c>
       <c r="B16" s="14"/>
       <c r="C16" s="14" t="s">
-        <v>214</v>
+        <v>159</v>
       </c>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
     </row>
     <row r="17" spans="1:5" ht="24">
       <c r="A17" s="14" t="s">
-        <v>244</v>
+        <v>189</v>
       </c>
       <c r="B17" s="14"/>
       <c r="C17" s="14" t="s">
-        <v>247</v>
+        <v>192</v>
       </c>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
     </row>
     <row r="18" spans="1:5" ht="36">
       <c r="A18" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>249</v>
+        <v>194</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>250</v>
+        <v>195</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>249</v>
+        <v>194</v>
       </c>
       <c r="E18" s="14" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="36">
       <c r="A19" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>249</v>
+        <v>194</v>
       </c>
       <c r="C19" s="14" t="s">
         <v>119</v>
       </c>
       <c r="D19" s="14" t="s">
-        <v>249</v>
+        <v>194</v>
       </c>
       <c r="E19" s="14" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="36">
       <c r="A20" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>249</v>
+        <v>194</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>251</v>
+        <v>196</v>
       </c>
       <c r="D20" s="14" t="s">
-        <v>249</v>
+        <v>194</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="24">
       <c r="A21" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>252</v>
+        <v>197</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>233</v>
+        <v>178</v>
       </c>
       <c r="D21" s="14"/>
       <c r="E21" s="14" t="s">
-        <v>235</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="24">
       <c r="A22" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>227</v>
+        <v>172</v>
       </c>
       <c r="C22" s="14" t="s">
-        <v>253</v>
+        <v>198</v>
       </c>
       <c r="D22" s="14"/>
       <c r="E22" s="14" t="s">
-        <v>235</v>
+        <v>180</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>254</v>
+        <v>199</v>
       </c>
       <c r="C23" s="14" t="s">
-        <v>255</v>
+        <v>200</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>254</v>
+        <v>199</v>
       </c>
       <c r="E23" s="14" t="s">
-        <v>235</v>
+        <v>180</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="36">
       <c r="A24" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>256</v>
+        <v>201</v>
       </c>
       <c r="C24" t="s">
-        <v>257</v>
+        <v>202</v>
       </c>
       <c r="D24" s="14" t="s">
-        <v>254</v>
+        <v>199</v>
       </c>
       <c r="E24" s="14" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="36">
       <c r="A25" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>258</v>
+        <v>203</v>
       </c>
       <c r="C25" t="s">
-        <v>259</v>
+        <v>204</v>
       </c>
       <c r="D25" s="14" t="s">
-        <v>254</v>
+        <v>199</v>
       </c>
       <c r="E25" s="14" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="36">
       <c r="A26" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>260</v>
+        <v>205</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>261</v>
+        <v>206</v>
       </c>
       <c r="D26" s="14" t="s">
-        <v>254</v>
+        <v>199</v>
       </c>
       <c r="E26" s="14" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="36">
       <c r="A27" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>262</v>
+        <v>207</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>263</v>
+        <v>208</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>254</v>
+        <v>199</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="60">
       <c r="A28" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>264</v>
+        <v>209</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>265</v>
+        <v>210</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>254</v>
+        <v>199</v>
       </c>
       <c r="E28" s="14" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="36">
       <c r="A29" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>266</v>
+        <v>211</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>267</v>
+        <v>212</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>254</v>
+        <v>199</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="48">
       <c r="A30" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>268</v>
+        <v>213</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>269</v>
+        <v>214</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>254</v>
+        <v>199</v>
       </c>
       <c r="E30" s="14" t="s">
-        <v>238</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="24">
       <c r="A31" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>271</v>
+        <v>216</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>272</v>
+        <v>217</v>
       </c>
       <c r="E31" s="14" t="s">
         <v>32</v>
@@ -6495,16 +6152,16 @@
     </row>
     <row r="32" spans="1:5" ht="36">
       <c r="A32" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C32" s="14" t="s">
-        <v>274</v>
+        <v>219</v>
       </c>
       <c r="D32" s="14" t="s">
-        <v>275</v>
+        <v>220</v>
       </c>
       <c r="E32" s="14" t="s">
         <v>32</v>
@@ -6512,16 +6169,16 @@
     </row>
     <row r="33" spans="1:5" ht="24">
       <c r="A33" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>276</v>
+        <v>221</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>277</v>
+        <v>222</v>
       </c>
       <c r="E33" s="14" t="s">
         <v>27</v>
@@ -6529,16 +6186,16 @@
     </row>
     <row r="34" spans="1:5">
       <c r="A34" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>278</v>
+        <v>223</v>
       </c>
       <c r="D34" s="14" t="s">
-        <v>277</v>
+        <v>222</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>27</v>
@@ -6546,16 +6203,16 @@
     </row>
     <row r="35" spans="1:5">
       <c r="A35" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>279</v>
+        <v>224</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>280</v>
+        <v>225</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>277</v>
+        <v>222</v>
       </c>
       <c r="E35" s="14" t="s">
         <v>27</v>
@@ -6563,16 +6220,16 @@
     </row>
     <row r="36" spans="1:5" ht="36">
       <c r="A36" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>281</v>
+        <v>226</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>282</v>
+        <v>227</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>281</v>
+        <v>226</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>35</v>
@@ -6580,16 +6237,16 @@
     </row>
     <row r="37" spans="1:5" ht="36">
       <c r="A37" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B37" s="14" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>283</v>
+        <v>228</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>284</v>
+        <v>229</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>35</v>
@@ -6597,16 +6254,16 @@
     </row>
     <row r="38" spans="1:5" ht="36">
       <c r="A38" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C38" s="17" t="s">
-        <v>285</v>
+        <v>230</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>286</v>
+        <v>231</v>
       </c>
       <c r="E38" s="14" t="s">
         <v>35</v>
@@ -6614,16 +6271,16 @@
     </row>
     <row r="39" spans="1:5">
       <c r="A39" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C39" s="17" t="s">
-        <v>287</v>
+        <v>232</v>
       </c>
       <c r="D39" s="17" t="s">
-        <v>286</v>
+        <v>231</v>
       </c>
       <c r="E39" s="14" t="s">
         <v>35</v>
@@ -6631,16 +6288,16 @@
     </row>
     <row r="40" spans="1:5" ht="36">
       <c r="A40" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C40" s="17" t="s">
-        <v>288</v>
+        <v>233</v>
       </c>
       <c r="D40" s="17" t="s">
-        <v>289</v>
+        <v>234</v>
       </c>
       <c r="E40" s="14" t="s">
         <v>35</v>
@@ -6648,303 +6305,303 @@
     </row>
     <row r="41" spans="1:5" ht="48">
       <c r="A41" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>290</v>
+        <v>235</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>291</v>
+        <v>237</v>
       </c>
     </row>
     <row r="42" spans="1:5" ht="36">
       <c r="A42" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C42" s="14" t="s">
-        <v>292</v>
+        <v>238</v>
       </c>
       <c r="D42" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>291</v>
+        <v>237</v>
       </c>
     </row>
     <row r="43" spans="1:5" ht="24">
       <c r="A43" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B43" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>293</v>
+        <v>239</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>294</v>
+        <v>240</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>295</v>
+        <v>241</v>
       </c>
       <c r="C44" s="14" t="s">
-        <v>278</v>
+        <v>223</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E44" s="14" t="s">
-        <v>294</v>
+        <v>240</v>
       </c>
     </row>
     <row r="45" spans="1:5" ht="24">
       <c r="A45" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>296</v>
+        <v>242</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>297</v>
+        <v>243</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="24">
       <c r="A46" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B46" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C46" s="14" t="s">
-        <v>298</v>
+        <v>244</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E46" s="14" t="s">
-        <v>297</v>
+        <v>243</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="24">
       <c r="A47" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>299</v>
+        <v>245</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>300</v>
+        <v>246</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>301</v>
+        <v>247</v>
       </c>
       <c r="D48" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E48" s="14" t="s">
-        <v>300</v>
+        <v>246</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="24">
       <c r="A49" s="14" t="s">
+        <v>193</v>
+      </c>
+      <c r="B49" s="17" t="s">
+        <v>215</v>
+      </c>
+      <c r="C49" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="B49" s="17" t="s">
-        <v>270</v>
-      </c>
-      <c r="C49" s="14" t="s">
-        <v>302</v>
-      </c>
       <c r="D49" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>303</v>
+        <v>249</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="24">
       <c r="A50" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B50" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C50" s="14" t="s">
-        <v>304</v>
+        <v>250</v>
       </c>
       <c r="D50" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E50" s="14" t="s">
-        <v>303</v>
+        <v>249</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="24">
       <c r="A51" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>305</v>
+        <v>251</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>306</v>
+        <v>252</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C52" s="14" t="s">
-        <v>307</v>
+        <v>253</v>
       </c>
       <c r="D52" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E52" s="14" t="s">
-        <v>306</v>
+        <v>252</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="24">
       <c r="A53" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B53" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>308</v>
+        <v>254</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>171</v>
+        <v>255</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="24">
       <c r="A54" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>309</v>
+        <v>256</v>
       </c>
       <c r="D54" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E54" s="14" t="s">
-        <v>310</v>
+        <v>257</v>
       </c>
     </row>
     <row r="55" spans="1:5" ht="24">
       <c r="A55" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>311</v>
+        <v>258</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>310</v>
+        <v>257</v>
       </c>
     </row>
     <row r="56" spans="1:5" ht="24">
       <c r="A56" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C56" s="14" t="s">
-        <v>308</v>
+        <v>254</v>
       </c>
       <c r="D56" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E56" s="14" t="s">
-        <v>312</v>
+        <v>259</v>
       </c>
     </row>
     <row r="57" spans="1:5" ht="24">
       <c r="A57" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B57" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>313</v>
+        <v>260</v>
       </c>
       <c r="D57" s="14"/>
       <c r="E57" s="14" t="s">
-        <v>314</v>
+        <v>261</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="36">
       <c r="A58" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B58" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C58" s="14" t="s">
-        <v>315</v>
+        <v>262</v>
       </c>
       <c r="D58" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E58" s="14" t="s">
         <v>38</v>
@@ -6952,16 +6609,16 @@
     </row>
     <row r="59" spans="1:5" ht="24">
       <c r="A59" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B59" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>316</v>
+        <v>263</v>
       </c>
       <c r="D59" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E59" s="14" t="s">
         <v>38</v>
@@ -6969,16 +6626,16 @@
     </row>
     <row r="60" spans="1:5" ht="24">
       <c r="A60" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B60" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C60" s="14" t="s">
-        <v>317</v>
+        <v>264</v>
       </c>
       <c r="D60" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E60" s="14" t="s">
         <v>48</v>
@@ -6986,16 +6643,16 @@
     </row>
     <row r="61" spans="1:5" ht="24">
       <c r="A61" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B61" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>318</v>
+        <v>265</v>
       </c>
       <c r="D61" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E61" s="14" t="s">
         <v>48</v>
@@ -7003,36 +6660,36 @@
     </row>
     <row r="62" spans="1:5">
       <c r="A62" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B62" s="17" t="s">
-        <v>270</v>
+        <v>215</v>
       </c>
       <c r="C62" s="14" t="s">
-        <v>319</v>
+        <v>266</v>
       </c>
       <c r="D62" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E62" s="33" t="s">
-        <v>320</v>
+        <v>267</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63" s="14" t="s">
-        <v>248</v>
+        <v>193</v>
       </c>
       <c r="B63" s="17" t="s">
-        <v>273</v>
+        <v>218</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>307</v>
+        <v>253</v>
       </c>
       <c r="D63" s="14" t="s">
-        <v>185</v>
+        <v>236</v>
       </c>
       <c r="E63" s="33" t="s">
-        <v>320</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -7056,71 +6713,71 @@
   <sheetData>
     <row r="1" spans="1:7" ht="42" customHeight="1">
       <c r="A1" s="9" t="s">
-        <v>321</v>
+        <v>268</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>322</v>
+        <v>269</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>323</v>
+        <v>270</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>324</v>
+        <v>271</v>
       </c>
       <c r="E1" s="9" t="s">
-        <v>325</v>
+        <v>272</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>326</v>
+        <v>273</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>327</v>
+        <v>274</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="14.25" customHeight="1">
       <c r="A2" s="13" t="s">
-        <v>328</v>
+        <v>275</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>329</v>
+        <v>276</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>329</v>
+        <v>276</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>329</v>
+        <v>276</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>329</v>
+        <v>276</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>329</v>
+        <v>276</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>329</v>
+        <v>276</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="35.1" customHeight="1">
       <c r="A3" s="18" t="s">
-        <v>330</v>
+        <v>277</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="C3" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="D3" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
       <c r="E3" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="23.85" customHeight="1">
@@ -7128,137 +6785,137 @@
         <v>89</v>
       </c>
       <c r="B4" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="C4" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="35.1" customHeight="1">
       <c r="A5" s="18" t="s">
-        <v>335</v>
+        <v>282</v>
       </c>
       <c r="B5" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="C5" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="F5" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="G5" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="23.85" customHeight="1">
       <c r="A6" s="18" t="s">
-        <v>336</v>
+        <v>283</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="D6" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="E6" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="F6" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="35.1" customHeight="1">
       <c r="A7" s="18" t="s">
-        <v>337</v>
+        <v>284</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
       <c r="E7" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="G7" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="23.85" customHeight="1">
       <c r="A8" s="18" t="s">
-        <v>338</v>
+        <v>285</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="D8" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="35.1" customHeight="1">
       <c r="A9" s="18" t="s">
-        <v>339</v>
+        <v>286</v>
       </c>
       <c r="B9" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="C9" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="D9" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="E9" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="G9" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="23.85" customHeight="1">
@@ -7266,68 +6923,68 @@
         <v>84</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
       <c r="E10" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="G10" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="35.1" customHeight="1">
       <c r="A11" s="18" t="s">
-        <v>340</v>
+        <v>287</v>
       </c>
       <c r="B11" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
       <c r="E11" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="G11" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="35.1" customHeight="1">
       <c r="A12" s="18" t="s">
-        <v>341</v>
+        <v>288</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>331</v>
+        <v>278</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>333</v>
+        <v>280</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>332</v>
+        <v>279</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>334</v>
+        <v>281</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="14.25" customHeight="1">
@@ -7341,19 +6998,19 @@
     </row>
     <row r="14" spans="1:7" ht="27.75" customHeight="1">
       <c r="A14" s="18" t="s">
-        <v>342</v>
+        <v>289</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>343</v>
+        <v>290</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>344</v>
+        <v>291</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>345</v>
+        <v>292</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>346</v>
+        <v>293</v>
       </c>
       <c r="F14" s="17"/>
       <c r="G14" s="17"/>
@@ -7377,21 +7034,21 @@
   <sheetData>
     <row r="1" spans="1:4" ht="14.25" customHeight="1">
       <c r="A1" s="9" t="s">
-        <v>347</v>
+        <v>294</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>348</v>
+        <v>295</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>349</v>
+        <v>296</v>
       </c>
       <c r="D1" s="9" t="s">
-        <v>350</v>
+        <v>297</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="22.35" customHeight="1">
       <c r="A2" s="13" t="s">
-        <v>351</v>
+        <v>298</v>
       </c>
       <c r="B2" s="13">
         <v>8</v>
@@ -7406,7 +7063,7 @@
     </row>
     <row r="3" spans="1:4" ht="23.85" customHeight="1">
       <c r="A3" s="18" t="s">
-        <v>352</v>
+        <v>299</v>
       </c>
       <c r="B3" s="14">
         <v>67</v>
@@ -7421,7 +7078,7 @@
     </row>
     <row r="4" spans="1:4" ht="35.1" customHeight="1">
       <c r="A4" s="18" t="s">
-        <v>353</v>
+        <v>300</v>
       </c>
       <c r="B4" s="14">
         <v>18</v>
@@ -7436,7 +7093,7 @@
     </row>
     <row r="5" spans="1:4" ht="35.1" customHeight="1">
       <c r="A5" s="18" t="s">
-        <v>354</v>
+        <v>301</v>
       </c>
       <c r="B5" s="14">
         <v>78</v>
@@ -7457,14 +7114,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="25b7c34c-a120-4ac3-ab60-c6bebc005a32">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2aea894b-94ad-406a-ad4e-500caf6a56d3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7663,16 +7318,18 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="25b7c34c-a120-4ac3-ab60-c6bebc005a32">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="2aea894b-94ad-406a-ad4e-500caf6a56d3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07A6E785-FFA4-4B45-919B-A658CFA9E29F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2FB2B9C-EC1C-4F74-BCCE-02A14630346E}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -7680,5 +7337,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2FB2B9C-EC1C-4F74-BCCE-02A14630346E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{07A6E785-FFA4-4B45-919B-A658CFA9E29F}"/>
 </file>
</xml_diff>